<commit_message>
IPO analysis: Royal Chain Limited (DRHP screen) + first filing scan
- companies/royal-chain-ltd: facts.json (restated figures with page cites),
  note.md, meta.json and the three generated workbooks. Call: Screen only,
  leaning Avoid at or above the Rs 147.33 pre-IPO reference.
- data/queue.json: eight further SEBI filings from 30-Sep/01-Oct queued;
  sources.json: SEBI listing verified, NSE bot-protection noted.
- toolkit: Quick Metrics now shows a metric blank (data gap) when a
  single-period input is blank, instead of computing it as zero.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GZaYU1Te5uSbV595LWtnFL
</commit_message>
<xml_diff>
--- a/ipo-analysis/templates/01_DRHP_Screening_Checklist.xlsx
+++ b/ipo-analysis/templates/01_DRHP_Screening_Checklist.xlsx
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="C33" s="16">
-        <f>SUM($C$11:$E$11)/SUM($C$10:$E$10)</f>
+        <f>IF(OR(ISBLANK($E$10),ISBLANK($E$11)),"",SUM($C$11:$E$11)/SUM($C$10:$E$10))</f>
         <v/>
       </c>
       <c r="D33" s="15" t="n">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="C34" s="16">
-        <f>SUM($C$8:$E$8)/SUM($C$7:$E$7)</f>
+        <f>IF(OR(ISBLANK($E$7),ISBLANK($E$8)),"",SUM($C$8:$E$8)/SUM($C$7:$E$7))</f>
         <v/>
       </c>
       <c r="D34" s="15" t="n">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="C35" s="16">
-        <f>$E$9/($E$8+$E$9)</f>
+        <f>IF(OR(ISBLANK($E$8),ISBLANK($E$9)),"",$E$9/($E$8+$E$9))</f>
         <v/>
       </c>
       <c r="D35" s="15" t="n">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="C36" s="16">
-        <f>$E$6/$E$7</f>
+        <f>IF(OR(ISBLANK($E$6),ISBLANK($E$7)),"",$E$6/$E$7)</f>
         <v/>
       </c>
       <c r="D36" s="15" t="n">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="C37" s="16">
-        <f>$E$12/$E$5</f>
+        <f>IF(OR(ISBLANK($E$12),ISBLANK($E$5)),"",$E$12/$E$5)</f>
         <v/>
       </c>
       <c r="D37" s="15" t="n">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="C38" s="16">
-        <f>$E$13/$E$14</f>
+        <f>IF(OR(ISBLANK($E$13),ISBLANK($E$14)),"",$E$13/$E$14)</f>
         <v/>
       </c>
       <c r="D38" s="15" t="n">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="C39" s="16">
-        <f>IFERROR(($E$12-$D$12)/($E$5-$D$5),"")</f>
+        <f>IF(OR(ISBLANK($E$12),ISBLANK($E$5)),"",IFERROR(($E$12-$D$12)/($E$5-$D$5),""))</f>
         <v/>
       </c>
       <c r="D39" s="15" t="n">
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="C40" s="16">
-        <f>$E$23</f>
+        <f>IF(OR(ISBLANK($E$23)),"",$E$23)</f>
         <v/>
       </c>
       <c r="D40" s="15" t="n">
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="C41" s="16">
-        <f>$E$24</f>
+        <f>IF(OR(ISBLANK($E$24)),"",$E$24)</f>
         <v/>
       </c>
       <c r="D41" s="15" t="n">
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="C42" s="16">
-        <f>$E$25</f>
+        <f>IF(OR(ISBLANK($E$25)),"",$E$25)</f>
         <v/>
       </c>
       <c r="D42" s="15" t="n">
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="C43" s="16">
-        <f>$E$26</f>
+        <f>IF(OR(ISBLANK($E$26)),"",$E$26)</f>
         <v/>
       </c>
       <c r="D43" s="15" t="n">
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="C44" s="16">
-        <f>$E$18/$E$14</f>
+        <f>IF(OR(ISBLANK($E$14),ISBLANK($E$18)),"",$E$18/$E$14)</f>
         <v/>
       </c>
       <c r="D44" s="15" t="n">
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="C45" s="16">
-        <f>$E$19/$E$14</f>
+        <f>IF(OR(ISBLANK($E$14),ISBLANK($E$19)),"",$E$19/$E$14)</f>
         <v/>
       </c>
       <c r="D45" s="15" t="n">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="C46" s="17">
-        <f>$E$20</f>
+        <f>IF(OR(ISBLANK($E$20)),"",$E$20)</f>
         <v/>
       </c>
       <c r="D46" s="14" t="n">
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="C47" s="18">
-        <f>$E$15/$E$5*365</f>
+        <f>IF(OR(ISBLANK($E$15),ISBLANK($E$5)),"",$E$15/$E$5*365)</f>
         <v/>
       </c>
       <c r="D47" s="19" t="n">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="C48" s="18">
-        <f>$E$16/$E$5*365</f>
+        <f>IF(OR(ISBLANK($E$16),ISBLANK($E$5)),"",$E$16/$E$5*365)</f>
         <v/>
       </c>
       <c r="D48" s="19" t="n">
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="C49" s="16">
-        <f>($E$15+$E$16-$E$17)/$E$5</f>
+        <f>IF(OR(ISBLANK($E$15),ISBLANK($E$16),ISBLANK($E$17),ISBLANK($E$5)),"",($E$15+$E$16-$E$17)/$E$5)</f>
         <v/>
       </c>
       <c r="D49" s="15" t="n">
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="C50" s="20">
-        <f>(($E$15+$E$16-$E$17)-($D$15+$D$16-$D$17))/($E$5-$D$5)</f>
+        <f>IF(OR(ISBLANK($E$15),ISBLANK($E$16),ISBLANK($E$17),ISBLANK($E$5)),"",(($E$15+$E$16-$E$17)-($D$15+$D$16-$D$17))/($E$5-$D$5))</f>
         <v/>
       </c>
       <c r="D50" s="21" t="n">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="C51" s="16">
-        <f>$E$10/$E$14</f>
+        <f>IF(OR(ISBLANK($E$10),ISBLANK($E$14)),"",$E$10/$E$14)</f>
         <v/>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="C52" s="16">
-        <f>$E$10/($E$14+$E$27)</f>
+        <f>IF(OR(ISBLANK($E$10),ISBLANK($E$14),ISBLANK($E$27)),"",$E$10/($E$14+$E$27))</f>
         <v/>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="C53" s="22">
-        <f>$E$29/$E$28</f>
+        <f>IF(OR(ISBLANK($E$28),ISBLANK($E$29)),"",$E$29/$E$28)</f>
         <v/>
       </c>
       <c r="D53" s="23" t="n">

</xml_diff>